<commit_message>
ingesta: snapshot 2026-07-28 18:20 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-07-28/Temp-max-julio-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-07-28/Temp-max-julio-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D029CB-7DFB-427D-9C10-27249A222173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0130718-98BB-445C-8536-09BA215828CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9502,14 +9502,16 @@
       <c r="AD5" s="57">
         <v>31.7</v>
       </c>
-      <c r="AE5" s="57"/>
+      <c r="AE5" s="57">
+        <v>31.3</v>
+      </c>
       <c r="AF5" s="57"/>
       <c r="AG5" s="57"/>
       <c r="AH5" s="57"/>
       <c r="AI5" s="57"/>
       <c r="AJ5" s="37">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>31.7</v>
+        <v>31.3</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9527,11 +9529,11 @@
       </c>
       <c r="AO5" s="23">
         <f>IF(COUNTIF(E5:AI5,"&gt;0")&gt;=15,AVERAGE(E5:AI5),"")</f>
-        <v>31.065384615384623</v>
+        <v>31.07407407407408</v>
       </c>
       <c r="AP5" s="23">
         <f>IF(AN5&gt;0,IFERROR(AO5-AN5,""),"")</f>
-        <v>0.8680128393763944</v>
+        <v>0.87670229806585098</v>
       </c>
     </row>
     <row r="6" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9625,14 +9627,16 @@
       <c r="AD6" s="57">
         <v>30.9</v>
       </c>
-      <c r="AE6" s="57"/>
+      <c r="AE6" s="57">
+        <v>31</v>
+      </c>
       <c r="AF6" s="57"/>
       <c r="AG6" s="57"/>
       <c r="AH6" s="57"/>
       <c r="AI6" s="57"/>
       <c r="AJ6" s="37">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>30.9</v>
+        <v>31</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
@@ -9650,11 +9654,11 @@
       </c>
       <c r="AO6" s="23">
         <f t="shared" ref="AO6:AO15" si="3">IF(COUNTIF(E6:AI6,"&gt;0")&gt;=15,AVERAGE(E6:AI6),"")</f>
-        <v>30.623076923076919</v>
+        <v>30.637037037037036</v>
       </c>
       <c r="AP6" s="23">
         <f t="shared" ref="AP6:AP48" si="4">IF(AN6&gt;0,IFERROR(AO6-AN6,""),"")</f>
-        <v>-3.1203473945421223E-2</v>
+        <v>-1.7243359985304352E-2</v>
       </c>
     </row>
     <row r="7" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9748,14 +9752,16 @@
       <c r="AD7" s="57">
         <v>34.6</v>
       </c>
-      <c r="AE7" s="57"/>
+      <c r="AE7" s="57">
+        <v>34.4</v>
+      </c>
       <c r="AF7" s="57"/>
       <c r="AG7" s="57"/>
       <c r="AH7" s="57"/>
       <c r="AI7" s="57"/>
       <c r="AJ7" s="37">
         <f t="shared" si="0"/>
-        <v>34.6</v>
+        <v>34.4</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9773,11 +9779,11 @@
       </c>
       <c r="AO7" s="23">
         <f t="shared" si="3"/>
-        <v>35.434615384615384</v>
+        <v>35.396296296296299</v>
       </c>
       <c r="AP7" s="23">
         <f t="shared" si="4"/>
-        <v>2.0685993770463114</v>
+        <v>2.0302802887272264</v>
       </c>
     </row>
     <row r="8" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9871,14 +9877,16 @@
       <c r="AD8" s="57">
         <v>33</v>
       </c>
-      <c r="AE8" s="57"/>
+      <c r="AE8" s="57">
+        <v>32.6</v>
+      </c>
       <c r="AF8" s="57"/>
       <c r="AG8" s="57"/>
       <c r="AH8" s="57"/>
       <c r="AI8" s="57"/>
       <c r="AJ8" s="37">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>32.6</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9896,11 +9904,11 @@
       </c>
       <c r="AO8" s="23">
         <f t="shared" si="3"/>
-        <v>33.165384615384617</v>
+        <v>33.144444444444446</v>
       </c>
       <c r="AP8" s="23">
         <f t="shared" si="4"/>
-        <v>0.91634160463192416</v>
+        <v>0.8954014336917524</v>
       </c>
     </row>
     <row r="9" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9994,14 +10002,16 @@
       <c r="AD9" s="57">
         <v>35</v>
       </c>
-      <c r="AE9" s="57"/>
+      <c r="AE9" s="57">
+        <v>32.9</v>
+      </c>
       <c r="AF9" s="57"/>
       <c r="AG9" s="57"/>
       <c r="AH9" s="57"/>
       <c r="AI9" s="57"/>
       <c r="AJ9" s="37">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>32.9</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -10019,11 +10029,11 @@
       </c>
       <c r="AO9" s="23">
         <f t="shared" si="3"/>
-        <v>33.819230769230771</v>
+        <v>33.785185185185185</v>
       </c>
       <c r="AP9" s="23">
         <f t="shared" si="4"/>
-        <v>0.72798463154692428</v>
+        <v>0.69393904750133828</v>
       </c>
     </row>
     <row r="10" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10117,14 +10127,16 @@
       <c r="AD10" s="57">
         <v>36.5</v>
       </c>
-      <c r="AE10" s="57"/>
+      <c r="AE10" s="57">
+        <v>35.1</v>
+      </c>
       <c r="AF10" s="57"/>
       <c r="AG10" s="57"/>
       <c r="AH10" s="57"/>
       <c r="AI10" s="57"/>
       <c r="AJ10" s="37">
         <f t="shared" si="0"/>
-        <v>36.5</v>
+        <v>35.1</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -10142,11 +10154,11 @@
       </c>
       <c r="AO10" s="23">
         <f t="shared" si="3"/>
-        <v>35.861538461538458</v>
+        <v>35.833333333333329</v>
       </c>
       <c r="AP10" s="23">
         <f t="shared" si="4"/>
-        <v>0.48130023387810184</v>
+        <v>0.45309510567297195</v>
       </c>
     </row>
     <row r="11" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10240,14 +10252,16 @@
       <c r="AD11" s="57">
         <v>38.4</v>
       </c>
-      <c r="AE11" s="57"/>
+      <c r="AE11" s="57">
+        <v>37.6</v>
+      </c>
       <c r="AF11" s="57"/>
       <c r="AG11" s="57"/>
       <c r="AH11" s="57"/>
       <c r="AI11" s="57"/>
       <c r="AJ11" s="37">
         <f t="shared" si="0"/>
-        <v>38.4</v>
+        <v>37.6</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -10265,11 +10279,11 @@
       </c>
       <c r="AO11" s="23">
         <f t="shared" si="3"/>
-        <v>38.053846153846145</v>
+        <v>38.037037037037031</v>
       </c>
       <c r="AP11" s="23">
         <f t="shared" si="4"/>
-        <v>2.5165620609975434</v>
+        <v>2.4997529441884296</v>
       </c>
     </row>
     <row r="12" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10363,14 +10377,16 @@
       <c r="AD12" s="57">
         <v>35</v>
       </c>
-      <c r="AE12" s="57"/>
+      <c r="AE12" s="57">
+        <v>33.200000000000003</v>
+      </c>
       <c r="AF12" s="57"/>
       <c r="AG12" s="57"/>
       <c r="AH12" s="57"/>
       <c r="AI12" s="57"/>
       <c r="AJ12" s="37">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10388,11 +10404,11 @@
       </c>
       <c r="AO12" s="23">
         <f t="shared" si="3"/>
-        <v>34.684615384615377</v>
+        <v>34.629629629629626</v>
       </c>
       <c r="AP12" s="23">
         <f t="shared" si="4"/>
-        <v>2.4959912384416398</v>
+        <v>2.4410054834558892</v>
       </c>
     </row>
     <row r="13" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10486,14 +10502,16 @@
       <c r="AD13" s="57">
         <v>35.200000000000003</v>
       </c>
-      <c r="AE13" s="57"/>
+      <c r="AE13" s="57">
+        <v>33</v>
+      </c>
       <c r="AF13" s="57"/>
       <c r="AG13" s="57"/>
       <c r="AH13" s="57"/>
       <c r="AI13" s="57"/>
       <c r="AJ13" s="37">
         <f t="shared" si="0"/>
-        <v>35.200000000000003</v>
+        <v>33</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10511,11 +10529,11 @@
       </c>
       <c r="AO13" s="23">
         <f t="shared" si="3"/>
-        <v>35.407692307692308</v>
+        <v>35.318518518518516</v>
       </c>
       <c r="AP13" s="23">
         <f t="shared" si="4"/>
-        <v>2.0259001929969713</v>
+        <v>1.9367264038231795</v>
       </c>
     </row>
     <row r="14" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10609,14 +10627,16 @@
       <c r="AD14" s="57">
         <v>33.299999999999997</v>
       </c>
-      <c r="AE14" s="57"/>
+      <c r="AE14" s="57">
+        <v>32.4</v>
+      </c>
       <c r="AF14" s="57"/>
       <c r="AG14" s="57"/>
       <c r="AH14" s="57"/>
       <c r="AI14" s="57"/>
       <c r="AJ14" s="37">
         <f t="shared" si="0"/>
-        <v>33.299999999999997</v>
+        <v>32.4</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10634,11 +10654,11 @@
       </c>
       <c r="AO14" s="23">
         <f t="shared" si="3"/>
-        <v>34.680769230769229</v>
+        <v>34.596296296296295</v>
       </c>
       <c r="AP14" s="23">
         <f t="shared" si="4"/>
-        <v>1.4558326315549976</v>
+        <v>1.3713596970820632</v>
       </c>
     </row>
     <row r="15" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10732,14 +10752,16 @@
       <c r="AD15" s="57">
         <v>30.4</v>
       </c>
-      <c r="AE15" s="57"/>
+      <c r="AE15" s="57">
+        <v>32.1</v>
+      </c>
       <c r="AF15" s="57"/>
       <c r="AG15" s="57"/>
       <c r="AH15" s="57"/>
       <c r="AI15" s="57"/>
       <c r="AJ15" s="37">
         <f t="shared" si="0"/>
-        <v>30.4</v>
+        <v>32.1</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10757,11 +10779,11 @@
       </c>
       <c r="AO15" s="23">
         <f t="shared" si="3"/>
-        <v>31.730769230769226</v>
+        <v>31.74444444444444</v>
       </c>
       <c r="AP15" s="23">
         <f t="shared" si="4"/>
-        <v>-4.5682253107237614E-3</v>
+        <v>9.1069883644898653E-3</v>
       </c>
     </row>
     <row r="16" spans="1:46" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -10904,14 +10926,16 @@
       <c r="AD17" s="57">
         <v>33.200000000000003</v>
       </c>
-      <c r="AE17" s="57"/>
+      <c r="AE17" s="57">
+        <v>33</v>
+      </c>
       <c r="AF17" s="57"/>
       <c r="AG17" s="57"/>
       <c r="AH17" s="57"/>
       <c r="AI17" s="57"/>
       <c r="AJ17" s="37">
         <f t="shared" si="0"/>
-        <v>33.200000000000003</v>
+        <v>33</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10929,11 +10953,11 @@
       </c>
       <c r="AO17" s="23">
         <f>IF(COUNTIF(E17:AI17,"&gt;0")&gt;=15,AVERAGE(E17:AI17),"")</f>
-        <v>34.119230769230768</v>
+        <v>34.077777777777776</v>
       </c>
       <c r="AP17" s="23">
         <f>IF(AN17&gt;0,IFERROR(AO17-AN17,""),"")</f>
-        <v>1.4452485667836115</v>
+        <v>1.4037955753306193</v>
       </c>
     </row>
     <row r="18" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11027,14 +11051,16 @@
       <c r="AD18" s="57">
         <v>27.2</v>
       </c>
-      <c r="AE18" s="57"/>
+      <c r="AE18" s="57">
+        <v>28.5</v>
+      </c>
       <c r="AF18" s="57"/>
       <c r="AG18" s="57"/>
       <c r="AH18" s="57"/>
       <c r="AI18" s="57"/>
       <c r="AJ18" s="37">
         <f t="shared" si="0"/>
-        <v>27.2</v>
+        <v>28.5</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -11052,11 +11078,11 @@
       </c>
       <c r="AO18" s="23">
         <f t="shared" ref="AO18:AO33" si="5">IF(COUNTIF(E18:AI18,"&gt;0")&gt;=15,AVERAGE(E18:AI18),"")</f>
-        <v>27.826923076923087</v>
+        <v>27.851851851851862</v>
       </c>
       <c r="AP18" s="23">
         <f t="shared" si="4"/>
-        <v>1.7670522229662176</v>
+        <v>1.7919809978949921</v>
       </c>
     </row>
     <row r="19" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11150,14 +11176,16 @@
       <c r="AD19" s="57">
         <v>35.799999999999997</v>
       </c>
-      <c r="AE19" s="57"/>
+      <c r="AE19" s="57">
+        <v>35.4</v>
+      </c>
       <c r="AF19" s="57"/>
       <c r="AG19" s="57"/>
       <c r="AH19" s="57"/>
       <c r="AI19" s="57"/>
       <c r="AJ19" s="37">
         <f t="shared" si="0"/>
-        <v>35.799999999999997</v>
+        <v>35.4</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -11175,11 +11203,11 @@
       </c>
       <c r="AO19" s="23">
         <f t="shared" si="5"/>
-        <v>33.776923076923069</v>
+        <v>33.837037037037028</v>
       </c>
       <c r="AP19" s="23">
         <f t="shared" si="4"/>
-        <v>0.52596067425342596</v>
+        <v>0.58607463436738527</v>
       </c>
     </row>
     <row r="20" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11273,14 +11301,16 @@
       <c r="AD20" s="57">
         <v>28</v>
       </c>
-      <c r="AE20" s="57"/>
+      <c r="AE20" s="57">
+        <v>30.9</v>
+      </c>
       <c r="AF20" s="57"/>
       <c r="AG20" s="57"/>
       <c r="AH20" s="57"/>
       <c r="AI20" s="57"/>
       <c r="AJ20" s="37">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>30.9</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -11298,11 +11328,11 @@
       </c>
       <c r="AO20" s="23">
         <f t="shared" si="5"/>
-        <v>30.130769230769236</v>
+        <v>30.159259259259262</v>
       </c>
       <c r="AP20" s="23">
         <f t="shared" si="4"/>
-        <v>1.4899646330680874</v>
+        <v>1.5184546615581134</v>
       </c>
     </row>
     <row r="21" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11396,14 +11426,16 @@
       <c r="AD21" s="57">
         <v>23.5</v>
       </c>
-      <c r="AE21" s="57"/>
+      <c r="AE21" s="57">
+        <v>24.1</v>
+      </c>
       <c r="AF21" s="57"/>
       <c r="AG21" s="57"/>
       <c r="AH21" s="57"/>
       <c r="AI21" s="57"/>
       <c r="AJ21" s="37">
         <f t="shared" si="0"/>
-        <v>23.5</v>
+        <v>24.1</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -11421,11 +11453,11 @@
       </c>
       <c r="AO21" s="23">
         <f t="shared" si="5"/>
-        <v>24.223076923076917</v>
+        <v>24.218518518518515</v>
       </c>
       <c r="AP21" s="23">
         <f t="shared" si="4"/>
-        <v>1.613573771426946</v>
+        <v>1.6090153668685439</v>
       </c>
     </row>
     <row r="22" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11587,14 +11619,16 @@
       <c r="AD23" s="57">
         <v>27.8</v>
       </c>
-      <c r="AE23" s="57"/>
+      <c r="AE23" s="57">
+        <v>27.6</v>
+      </c>
       <c r="AF23" s="57"/>
       <c r="AG23" s="57"/>
       <c r="AH23" s="57"/>
       <c r="AI23" s="57"/>
       <c r="AJ23" s="37">
         <f t="shared" si="0"/>
-        <v>27.8</v>
+        <v>27.6</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -11612,11 +11646,11 @@
       </c>
       <c r="AO23" s="23">
         <f t="shared" si="5"/>
-        <v>28.561538461538461</v>
+        <v>28.525925925925929</v>
       </c>
       <c r="AP23" s="23">
         <f t="shared" si="4"/>
-        <v>1.6931513647642618</v>
+        <v>1.6575388291517292</v>
       </c>
     </row>
     <row r="24" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11710,14 +11744,16 @@
       <c r="AD24" s="57">
         <v>27.8</v>
       </c>
-      <c r="AE24" s="57"/>
+      <c r="AE24" s="57">
+        <v>29.1</v>
+      </c>
       <c r="AF24" s="57"/>
       <c r="AG24" s="57"/>
       <c r="AH24" s="57"/>
       <c r="AI24" s="57"/>
       <c r="AJ24" s="37">
         <f t="shared" si="0"/>
-        <v>27.8</v>
+        <v>29.1</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -11735,11 +11771,11 @@
       </c>
       <c r="AO24" s="23">
         <f t="shared" si="5"/>
-        <v>29.450000000000003</v>
+        <v>29.43703703703704</v>
       </c>
       <c r="AP24" s="23">
         <f t="shared" si="4"/>
-        <v>1.1981758832565212</v>
+        <v>1.1852129202935586</v>
       </c>
     </row>
     <row r="25" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11833,14 +11869,16 @@
       <c r="AD25" s="57">
         <v>31.8</v>
       </c>
-      <c r="AE25" s="57"/>
+      <c r="AE25" s="57">
+        <v>33.9</v>
+      </c>
       <c r="AF25" s="57"/>
       <c r="AG25" s="57"/>
       <c r="AH25" s="57"/>
       <c r="AI25" s="57"/>
       <c r="AJ25" s="37">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>33.9</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11858,11 +11896,11 @@
       </c>
       <c r="AO25" s="23">
         <f t="shared" si="5"/>
-        <v>32.396153846153851</v>
+        <v>32.451851851851856</v>
       </c>
       <c r="AP25" s="23">
         <f t="shared" si="4"/>
-        <v>2.0202884529327818</v>
+        <v>2.075986458630787</v>
       </c>
     </row>
     <row r="26" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11956,14 +11994,16 @@
       <c r="AD26" s="57">
         <v>18.2</v>
       </c>
-      <c r="AE26" s="57"/>
+      <c r="AE26" s="57">
+        <v>20.2</v>
+      </c>
       <c r="AF26" s="57"/>
       <c r="AG26" s="57"/>
       <c r="AH26" s="57"/>
       <c r="AI26" s="57"/>
       <c r="AJ26" s="37">
         <f t="shared" si="0"/>
-        <v>18.2</v>
+        <v>20.2</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11981,11 +12021,11 @@
       </c>
       <c r="AO26" s="23">
         <f t="shared" si="5"/>
-        <v>19.661538461538463</v>
+        <v>19.681481481481484</v>
       </c>
       <c r="AP26" s="23">
         <f t="shared" si="4"/>
-        <v>1.1186668540951032</v>
+        <v>1.1386098740381243</v>
       </c>
     </row>
     <row r="27" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12077,14 +12117,16 @@
       <c r="AD27" s="57">
         <v>21.4</v>
       </c>
-      <c r="AE27" s="57"/>
+      <c r="AE27" s="57">
+        <v>20</v>
+      </c>
       <c r="AF27" s="57"/>
       <c r="AG27" s="57"/>
       <c r="AH27" s="57"/>
       <c r="AI27" s="57"/>
       <c r="AJ27" s="37">
         <f t="shared" si="0"/>
-        <v>21.4</v>
+        <v>20</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
@@ -12102,11 +12144,11 @@
       </c>
       <c r="AO27" s="23">
         <f t="shared" si="5"/>
-        <v>18.903999999999996</v>
+        <v>18.946153846153841</v>
       </c>
       <c r="AP27" s="23">
         <f t="shared" si="4"/>
-        <v>2.2219494558916075</v>
+        <v>2.2641033020454522</v>
       </c>
     </row>
     <row r="28" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12200,14 +12242,16 @@
       <c r="AD28" s="57">
         <v>30.8</v>
       </c>
-      <c r="AE28" s="57"/>
+      <c r="AE28" s="57">
+        <v>31.1</v>
+      </c>
       <c r="AF28" s="57"/>
       <c r="AG28" s="57"/>
       <c r="AH28" s="57"/>
       <c r="AI28" s="57"/>
       <c r="AJ28" s="37">
         <f t="shared" si="0"/>
-        <v>30.8</v>
+        <v>31.1</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -12225,11 +12269,11 @@
       </c>
       <c r="AO28" s="23">
         <f t="shared" si="5"/>
-        <v>31.934615384615388</v>
+        <v>31.903703703703709</v>
       </c>
       <c r="AP28" s="23">
         <f t="shared" si="4"/>
-        <v>1.4061627829592283</v>
+        <v>1.3752511020475495</v>
       </c>
     </row>
     <row r="29" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12389,36 +12433,38 @@
       <c r="AD30" s="57">
         <v>34.700000000000003</v>
       </c>
-      <c r="AE30" s="57"/>
+      <c r="AE30" s="57">
+        <v>37.299999999999997</v>
+      </c>
       <c r="AF30" s="57"/>
       <c r="AG30" s="57"/>
       <c r="AH30" s="57"/>
       <c r="AI30" s="57"/>
       <c r="AJ30" s="37">
         <f t="shared" si="0"/>
-        <v>34.700000000000003</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
-        <v>37.200000000000003</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="AL30" s="22">
         <v>38.6</v>
       </c>
       <c r="AM30" s="23">
         <f t="shared" si="2"/>
-        <v>-1.3999999999999986</v>
+        <v>-1.3000000000000043</v>
       </c>
       <c r="AN30" s="23">
         <v>33.74225089605735</v>
       </c>
       <c r="AO30" s="23">
         <f t="shared" si="5"/>
-        <v>34.807692307692314</v>
+        <v>34.900000000000006</v>
       </c>
       <c r="AP30" s="23">
         <f t="shared" si="4"/>
-        <v>1.0654414116349642</v>
+        <v>1.1577491039426562</v>
       </c>
     </row>
     <row r="31" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12512,14 +12558,16 @@
       <c r="AD31" s="57">
         <v>27.2</v>
       </c>
-      <c r="AE31" s="57"/>
+      <c r="AE31" s="57">
+        <v>27</v>
+      </c>
       <c r="AF31" s="57"/>
       <c r="AG31" s="57"/>
       <c r="AH31" s="57"/>
       <c r="AI31" s="57"/>
       <c r="AJ31" s="37">
         <f t="shared" si="0"/>
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -12537,11 +12585,11 @@
       </c>
       <c r="AO31" s="23">
         <f t="shared" si="5"/>
-        <v>27.25</v>
+        <v>27.24074074074074</v>
       </c>
       <c r="AP31" s="23">
         <f t="shared" si="4"/>
-        <v>1.8625751628793807</v>
+        <v>1.8533159036201212</v>
       </c>
     </row>
     <row r="32" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12635,14 +12683,16 @@
       <c r="AD32" s="57">
         <v>16.600000000000001</v>
       </c>
-      <c r="AE32" s="57"/>
+      <c r="AE32" s="57">
+        <v>17.8</v>
+      </c>
       <c r="AF32" s="57"/>
       <c r="AG32" s="57"/>
       <c r="AH32" s="57"/>
       <c r="AI32" s="57"/>
       <c r="AJ32" s="37">
         <f t="shared" si="0"/>
-        <v>16.600000000000001</v>
+        <v>17.8</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -12660,11 +12710,11 @@
       </c>
       <c r="AO32" s="23">
         <f t="shared" si="5"/>
-        <v>17.76923076923077</v>
+        <v>17.770370370370372</v>
       </c>
       <c r="AP32" s="23">
         <f t="shared" si="4"/>
-        <v>1.4396929959695193</v>
+        <v>1.4408325971091216</v>
       </c>
     </row>
     <row r="33" spans="1:47" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12758,14 +12808,16 @@
       <c r="AD33" s="57">
         <v>15.6</v>
       </c>
-      <c r="AE33" s="57"/>
+      <c r="AE33" s="57">
+        <v>14.6</v>
+      </c>
       <c r="AF33" s="57"/>
       <c r="AG33" s="57"/>
       <c r="AH33" s="57"/>
       <c r="AI33" s="57"/>
       <c r="AJ33" s="37">
         <f t="shared" si="0"/>
-        <v>15.6</v>
+        <v>14.6</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -12783,11 +12835,11 @@
       </c>
       <c r="AO33" s="23">
         <f t="shared" si="5"/>
-        <v>15.688461538461537</v>
+        <v>15.648148148148149</v>
       </c>
       <c r="AP33" s="23">
         <f t="shared" si="4"/>
-        <v>0.94384900601808752</v>
+        <v>0.90353561570469942</v>
       </c>
       <c r="AT33" s="15"/>
     </row>
@@ -12933,14 +12985,16 @@
       <c r="AD35" s="57">
         <v>28.2</v>
       </c>
-      <c r="AE35" s="57"/>
+      <c r="AE35" s="57">
+        <v>33.799999999999997</v>
+      </c>
       <c r="AF35" s="57"/>
       <c r="AG35" s="57"/>
       <c r="AH35" s="57"/>
       <c r="AI35" s="57"/>
       <c r="AJ35" s="37">
         <f t="shared" si="0"/>
-        <v>28.2</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -12958,11 +13012,11 @@
       </c>
       <c r="AO35" s="23">
         <f>IF(COUNTIF(E35:AI35,"&gt;0")&gt;=15,AVERAGE(E35:AI35),"")</f>
-        <v>31.776923076923076</v>
+        <v>31.851851851851848</v>
       </c>
       <c r="AP35" s="23">
         <f t="shared" si="4"/>
-        <v>0.70422722438851437</v>
+        <v>0.77915599931728607</v>
       </c>
       <c r="AT35" s="15"/>
     </row>
@@ -13177,14 +13231,16 @@
       <c r="AD38" s="57">
         <v>26.5</v>
       </c>
-      <c r="AE38" s="57"/>
+      <c r="AE38" s="57">
+        <v>30.6</v>
+      </c>
       <c r="AF38" s="57"/>
       <c r="AG38" s="57"/>
       <c r="AH38" s="57"/>
       <c r="AI38" s="57"/>
       <c r="AJ38" s="37">
         <f t="shared" si="0"/>
-        <v>26.5</v>
+        <v>30.6</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -13202,11 +13258,11 @@
       </c>
       <c r="AO38" s="23">
         <f>IF(COUNTIF(E38:AI38,"&gt;0")&gt;=15,AVERAGE(E38:AI38),"")</f>
-        <v>30.042307692307688</v>
+        <v>30.06296296296296</v>
       </c>
       <c r="AP38" s="23">
         <f t="shared" si="4"/>
-        <v>1.3281468915106842E-2</v>
+        <v>3.3936739570378904E-2</v>
       </c>
       <c r="AT38" s="15"/>
     </row>
@@ -13301,14 +13357,16 @@
       <c r="AD39" s="57">
         <v>29</v>
       </c>
-      <c r="AE39" s="57"/>
+      <c r="AE39" s="57">
+        <v>33.4</v>
+      </c>
       <c r="AF39" s="57"/>
       <c r="AG39" s="57"/>
       <c r="AH39" s="57"/>
       <c r="AI39" s="57"/>
       <c r="AJ39" s="37">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>33.4</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -13326,11 +13384,11 @@
       </c>
       <c r="AO39" s="23">
         <f t="shared" ref="AO39:AO48" si="7">IF(COUNTIF(E39:AI39,"&gt;0")&gt;=15,AVERAGE(E39:AI39),"")</f>
-        <v>31.426923076923078</v>
+        <v>31.5</v>
       </c>
       <c r="AP39" s="23">
         <f t="shared" si="4"/>
-        <v>0.58378996605915745</v>
+        <v>0.65686688913607938</v>
       </c>
       <c r="AT39" s="15"/>
     </row>
@@ -13425,14 +13483,16 @@
       <c r="AD40" s="57">
         <v>30.6</v>
       </c>
-      <c r="AE40" s="57"/>
+      <c r="AE40" s="57">
+        <v>31.2</v>
+      </c>
       <c r="AF40" s="57"/>
       <c r="AG40" s="57"/>
       <c r="AH40" s="57"/>
       <c r="AI40" s="57"/>
       <c r="AJ40" s="37">
         <f t="shared" si="0"/>
-        <v>30.6</v>
+        <v>31.2</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -13450,11 +13510,11 @@
       </c>
       <c r="AO40" s="23">
         <f t="shared" si="7"/>
-        <v>29.919230769230769</v>
+        <v>29.966666666666669</v>
       </c>
       <c r="AP40" s="23">
         <f t="shared" si="4"/>
-        <v>0.97168238213398794</v>
+        <v>1.0191182795698879</v>
       </c>
       <c r="AT40" s="15"/>
     </row>
@@ -13549,14 +13609,16 @@
       <c r="AD41" s="57">
         <v>28.2</v>
       </c>
-      <c r="AE41" s="57"/>
+      <c r="AE41" s="57">
+        <v>32.6</v>
+      </c>
       <c r="AF41" s="57"/>
       <c r="AG41" s="57"/>
       <c r="AH41" s="57"/>
       <c r="AI41" s="57"/>
       <c r="AJ41" s="37">
         <f t="shared" si="0"/>
-        <v>28.2</v>
+        <v>32.6</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="1"/>
@@ -13574,11 +13636,11 @@
       </c>
       <c r="AO41" s="23">
         <f t="shared" si="7"/>
-        <v>30.553846153846163</v>
+        <v>30.629629629629637</v>
       </c>
       <c r="AP41" s="23">
         <f t="shared" si="4"/>
-        <v>1.1875379101185715</v>
+        <v>1.2633213859020458</v>
       </c>
       <c r="AT41" s="15"/>
     </row>
@@ -13734,36 +13796,38 @@
       <c r="AD43" s="57">
         <v>32</v>
       </c>
-      <c r="AE43" s="57"/>
+      <c r="AE43" s="57">
+        <v>33.6</v>
+      </c>
       <c r="AF43" s="57"/>
       <c r="AG43" s="57"/>
       <c r="AH43" s="57"/>
       <c r="AI43" s="57"/>
       <c r="AJ43" s="37">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>33.6</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
-        <v>33.200000000000003</v>
+        <v>33.6</v>
       </c>
       <c r="AL43" s="22">
         <v>34.200000000000003</v>
       </c>
       <c r="AM43" s="23">
         <f t="shared" si="2"/>
-        <v>-1</v>
+        <v>-0.60000000000000142</v>
       </c>
       <c r="AN43" s="23">
         <v>30.061061827956991</v>
       </c>
       <c r="AO43" s="23">
         <f t="shared" si="7"/>
-        <v>31.173913043478262</v>
+        <v>31.275000000000002</v>
       </c>
       <c r="AP43" s="23">
         <f t="shared" si="4"/>
-        <v>1.1128512155212711</v>
+        <v>1.2139381720430116</v>
       </c>
       <c r="AT43" s="15"/>
     </row>
@@ -13856,14 +13920,16 @@
       <c r="AD44" s="29">
         <v>32.200000000000003</v>
       </c>
-      <c r="AE44" s="57"/>
+      <c r="AE44" s="57">
+        <v>32.299999999999997</v>
+      </c>
       <c r="AF44" s="57"/>
       <c r="AG44" s="57"/>
       <c r="AH44" s="57"/>
       <c r="AI44" s="57"/>
       <c r="AJ44" s="37">
         <f t="shared" si="0"/>
-        <v>32.200000000000003</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="1"/>
@@ -13881,11 +13947,11 @@
       </c>
       <c r="AO44" s="23">
         <f t="shared" si="7"/>
-        <v>31.251999999999999</v>
+        <v>31.292307692307688</v>
       </c>
       <c r="AP44" s="23">
         <f t="shared" si="4"/>
-        <v>2.2088127946395382</v>
+        <v>2.249120486947227</v>
       </c>
       <c r="AT44" s="15"/>
     </row>
@@ -13980,14 +14046,16 @@
       <c r="AD45" s="57">
         <v>30.2</v>
       </c>
-      <c r="AE45" s="57"/>
+      <c r="AE45" s="57">
+        <v>32.799999999999997</v>
+      </c>
       <c r="AF45" s="57"/>
       <c r="AG45" s="57"/>
       <c r="AH45" s="57"/>
       <c r="AI45" s="57"/>
       <c r="AJ45" s="37">
         <f t="shared" si="0"/>
-        <v>30.2</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -14005,11 +14073,11 @@
       </c>
       <c r="AO45" s="23">
         <f t="shared" si="7"/>
-        <v>30.607692307692318</v>
+        <v>30.688888888888897</v>
       </c>
       <c r="AP45" s="23">
         <f t="shared" si="4"/>
-        <v>1.0618759148134878</v>
+        <v>1.1430724960100669</v>
       </c>
       <c r="AT45" s="15"/>
     </row>
@@ -14243,14 +14311,16 @@
       <c r="AD48" s="57">
         <v>31.7</v>
       </c>
-      <c r="AE48" s="57"/>
+      <c r="AE48" s="57">
+        <v>29.7</v>
+      </c>
       <c r="AF48" s="57"/>
       <c r="AG48" s="57"/>
       <c r="AH48" s="57"/>
       <c r="AI48" s="57"/>
       <c r="AJ48" s="37">
         <f t="shared" si="0"/>
-        <v>31.7</v>
+        <v>29.7</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -14268,11 +14338,11 @@
       </c>
       <c r="AO48" s="23">
         <f t="shared" si="7"/>
-        <v>30.746153846153849</v>
+        <v>30.707407407407413</v>
       </c>
       <c r="AP48" s="23">
         <f t="shared" si="4"/>
-        <v>0.40362099071776925</v>
+        <v>0.36487455197133301</v>
       </c>
     </row>
     <row r="49" spans="5:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -27171,12 +27241,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -27186,6 +27250,12 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>